<commit_message>
fix(jd): 同步远程 Pull 后 Cookie 路径不一致（cookie.txt→sz_cookie.txt）
问题（2026-08-12 远程 Pull 后发现）：
- 远程把 .gitignore 改成排除 config/sz_cookie.txt（旧名 cookie.txt 取消保护）
- 但远程漏改两处代码仍指 config/cookie.txt，导致 Cookie 文件找不到
- 商智项目13（关键词分析）等所有商智业务跑不通

修复内容：
1. main.py 基类 JDBaseRequest 默认 Cookie 路径兜底：
   os.path.join(project_root, "config", "cookie.txt")
   → os.path.join(project_root, "config", "sz_cookie.txt")
   （防止 config.xlsx 未配置时找不到 Cookie）
2. config/config.xlsx 「全局配置」cookie文件路径：
   config/cookie.txt → config/sz_cookie.txt
   （与 .gitignore 新规则一致）

用户提示：
- 本地有 config/cookie.txt 的需手动重命名为 config/sz_cookie.txt
  （已完成此手动操作；Cookie 内容不变）

验收：
- 商智关键词分析月粒度（7 月）：300行×27列 跑通 ✅

注：远程 commit 漏改 config.xlsx 是上游 bug，本修复是项目13 商智关键词分析可用性的紧急兼容修复。
待远程下次同步时检查是否已统一改成 sz_cookie.txt。
</commit_message>
<xml_diff>
--- a/config/config.xlsx
+++ b/config/config.xlsx
@@ -1,12 +1,12 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" windowWidth="27945" windowHeight="12375" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="全局配置" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="全局配置" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="191029" calcMode="manual" fullCalcOnLoad="1"/>
@@ -1121,7 +1121,7 @@
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>config/cookie.txt</t>
+          <t>config/sz_cookie.txt</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">

</xml_diff>